<commit_message>
Added forget password feature with properties file
</commit_message>
<xml_diff>
--- a/src/test/resources/QuestionData.xlsx
+++ b/src/test/resources/QuestionData.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Automation-Project-main\com.ecom\src\test\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{759FACA3-F35B-4DA5-A133-275AD6E40B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CFA8E93-CA1C-4A83-A559-1310BBE3C238}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="20790" windowHeight="11820" xr2:uid="{4CFA8E93-CA1C-4A83-A559-1310BBE3C238}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -129,9 +125,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -169,7 +165,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -275,7 +271,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -417,7 +413,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -426,9 +422,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE044C57-7474-40BB-BDF3-AD977BF42002}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -442,7 +438,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>

</xml_diff>